<commit_message>
Add spatial-transfer reading map and append evidence to scientific guide
</commit_message>
<xml_diff>
--- a/results/ad-oxygen-literature-20261006/oxygen_response_review/spatial_gas_transfer/spatial_gas_transfer_cumulative.xlsx
+++ b/results/ad-oxygen-literature-20261006/oxygen_response_review/spatial_gas_transfer/spatial_gas_transfer_cumulative.xlsx
@@ -979,6 +979,16 @@
           <t>results/ad-oxygen-literature-20261006/omics_dataset_discovery/raw/NCBI/cfc7af329ca2b6a6948e25003e2b6ddc6f91b2e2dc3e867e63108f407191f658.body</t>
         </is>
       </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>A 产甲烷直接（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL5" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -1327,6 +1337,16 @@
           <t>results/ad-oxygen-literature-20261006/omics_dataset_discovery/raw/NCBI/cfc7af329ca2b6a6948e25003e2b6ddc6f91b2e2dc3e867e63108f407191f658.body</t>
         </is>
       </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>C 天然成像方法（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL8" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -1445,6 +1465,16 @@
       <c r="AC9" t="b">
         <v>0</v>
       </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>导航综述（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL9" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -2882,6 +2912,16 @@
           <t>results/ad-oxygen-literature-20261006/omics_dataset_discovery/raw/NCBI/1986329a541e64ec6ec832c62ee17bee05ca3f6c784fb52bd53d2341f1a1f8d9.body</t>
         </is>
       </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>A 产甲烷直接（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK27" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL27" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -3000,6 +3040,16 @@
       <c r="AC28" t="b">
         <v>0</v>
       </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>C DAMO/Anammox模型（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK28" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL28" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -4032,6 +4082,16 @@
       <c r="AC40" t="b">
         <v>0</v>
       </c>
+      <c r="AE40" t="inlineStr">
+        <is>
+          <t>C DAMO/Anammox传质参照（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK40" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL40" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -4776,6 +4836,16 @@
           <t>results/ad-oxygen-literature-20261006/omics_dataset_discovery/raw/NCBI/36328184af1a8747e4473dc767f2753f5f61f250c369017f68b452c5d63ba90a.body</t>
         </is>
       </c>
+      <c r="AE49" t="inlineStr">
+        <is>
+          <t>A 产甲烷直接（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK49" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL49" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -5371,6 +5441,16 @@
           <t>results/ad-oxygen-literature-20261006/omics_dataset_discovery/raw/NCBI/4c7b9de88dc3c2b30f7806e60e8ba11074b3948ba15c7089ac42c3b2eb226dd9.body</t>
         </is>
       </c>
+      <c r="AE56" t="inlineStr">
+        <is>
+          <t>A 互营共培养（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK56" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL56" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -5571,6 +5651,16 @@
       <c r="AC58" t="b">
         <v>0</v>
       </c>
+      <c r="AE58" t="inlineStr">
+        <is>
+          <t>A CO2甲烷化生物膜（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK58" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL58" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -5776,6 +5866,16 @@
           <t>results/ad-oxygen-literature-20261006/omics_dataset_discovery/raw/NCBI/4c7b9de88dc3c2b30f7806e60e8ba11074b3948ba15c7089ac42c3b2eb226dd9.body</t>
         </is>
       </c>
+      <c r="AE60" t="inlineStr">
+        <is>
+          <t>A 产甲烷直接（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK60" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL60" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -6202,6 +6302,16 @@
       <c r="AC65" t="b">
         <v>0</v>
       </c>
+      <c r="AE65" t="inlineStr">
+        <is>
+          <t>C 甲烷氧化脱氮膜（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK65" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL65" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -6551,6 +6661,16 @@
       <c r="AC69" t="b">
         <v>0</v>
       </c>
+      <c r="AE69" t="inlineStr">
+        <is>
+          <t>C 甲烷氧化方法（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK69" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL69" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -7218,6 +7338,16 @@
           <t>results/ad-oxygen-literature-20261006/omics_dataset_discovery/raw/NCBI/863e1adc64fc7079316bfb5f12b86c02fb0085e72978511e95d4520981794eb8.body</t>
         </is>
       </c>
+      <c r="AE77" t="inlineStr">
+        <is>
+          <t>A 产甲烷AD载体（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK77" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL77" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -8337,6 +8467,16 @@
       <c r="AC91" t="b">
         <v>0</v>
       </c>
+      <c r="AE91" t="inlineStr">
+        <is>
+          <t>B 界面电子传递背景（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK91" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL91" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -9505,6 +9645,16 @@
       <c r="AC104" t="b">
         <v>0</v>
       </c>
+      <c r="AE104" t="inlineStr">
+        <is>
+          <t>C DAMO/Anammox（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK104" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL104" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -9705,6 +9855,16 @@
       </c>
       <c r="AC106" t="b">
         <v>0</v>
+      </c>
+      <c r="AE106" t="inlineStr">
+        <is>
+          <t>C Anammox方法参照（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK106" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
       </c>
       <c r="AL106" t="inlineStr">
         <is>
@@ -11229,6 +11389,16 @@
       <c r="AC124" t="b">
         <v>0</v>
       </c>
+      <c r="AE124" t="inlineStr">
+        <is>
+          <t>C 脱氮生物膜方法（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK124" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL124" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -14141,6 +14311,16 @@
       <c r="AC157" t="b">
         <v>0</v>
       </c>
+      <c r="AE157" t="inlineStr">
+        <is>
+          <t>C 天然/方法参照（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK157" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL157" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -14678,6 +14858,16 @@
       </c>
       <c r="AC163" t="b">
         <v>0</v>
+      </c>
+      <c r="AE163" t="inlineStr">
+        <is>
+          <t>C 下水道生物膜（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK163" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
       </c>
       <c r="AL163" t="inlineStr">
         <is>
@@ -16695,6 +16885,16 @@
       <c r="AC187" t="b">
         <v>0</v>
       </c>
+      <c r="AE187" t="inlineStr">
+        <is>
+          <t>C 其他生物膜方法（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK187" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL187" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -17274,6 +17474,16 @@
       <c r="AC194" t="b">
         <v>0</v>
       </c>
+      <c r="AE194" t="inlineStr">
+        <is>
+          <t>A 膜气体模型（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK194" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL194" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -18201,6 +18411,16 @@
       <c r="AC203" t="b">
         <v>0</v>
       </c>
+      <c r="AE203" t="inlineStr">
+        <is>
+          <t>A AD气泡处理（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK203" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL203" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -18489,6 +18709,16 @@
       <c r="AC206" t="b">
         <v>0</v>
       </c>
+      <c r="AE206" t="inlineStr">
+        <is>
+          <t>C 好氧颗粒控制参照（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK206" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL206" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -18611,6 +18841,16 @@
       </c>
       <c r="AC207" t="b">
         <v>0</v>
+      </c>
+      <c r="AE207" t="inlineStr">
+        <is>
+          <t>A AD混合干预（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK207" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
       </c>
       <c r="AL207" t="inlineStr">
         <is>
@@ -19040,6 +19280,16 @@
       <c r="AC211" t="b">
         <v>0</v>
       </c>
+      <c r="AE211" t="inlineStr">
+        <is>
+          <t>A 脱硫模型导航（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK211" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL211" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -19237,6 +19487,16 @@
       <c r="AC213" t="b">
         <v>0</v>
       </c>
+      <c r="AE213" t="inlineStr">
+        <is>
+          <t>导航综述（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK213" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL213" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -19836,6 +20096,16 @@
       <c r="AC220" t="b">
         <v>0</v>
       </c>
+      <c r="AE220" t="inlineStr">
+        <is>
+          <t>导航综述（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK220" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL220" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -20133,6 +20403,16 @@
       <c r="AC223" t="b">
         <v>0</v>
       </c>
+      <c r="AE223" t="inlineStr">
+        <is>
+          <t>A AD相关膜生物膜（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK223" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL223" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -20256,6 +20536,16 @@
       <c r="AC224" t="b">
         <v>0</v>
       </c>
+      <c r="AE224" t="inlineStr">
+        <is>
+          <t>A 产甲烷直接（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK224" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
+      </c>
       <c r="AL224" t="inlineStr">
         <is>
           <t>空值表示本轮尚未核实，不能推断原文未报告</t>
@@ -20784,6 +21074,16 @@
       </c>
       <c r="AC230" t="b">
         <v>0</v>
+      </c>
+      <c r="AE230" t="inlineStr">
+        <is>
+          <t>导航综述（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK230" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
       </c>
       <c r="AL230" t="inlineStr">
         <is>
@@ -20896,6 +21196,16 @@
       </c>
       <c r="AC231" t="b">
         <v>0</v>
+      </c>
+      <c r="AE231" t="inlineStr">
+        <is>
+          <t>待核实研究线索（详见actual_finding和decision_reason；具体条件未核字段留空）</t>
+        </is>
+      </c>
+      <c r="AK231" t="inlineStr">
+        <is>
+          <t>完整缓存摘要；具体正文位置尚待核实</t>
+        </is>
       </c>
       <c r="AL231" t="inlineStr">
         <is>

</xml_diff>